<commit_message>
Order dataset record dates chronologically
</commit_message>
<xml_diff>
--- a/public/templates/upload_new_datasets_template.xlsx
+++ b/public/templates/upload_new_datasets_template.xlsx
@@ -540,10 +540,10 @@
         <v>8</v>
       </c>
       <c r="P1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q1" t="s">
         <v>35</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>37</v>
       </c>
       <c r="R1" t="s">
         <v>39</v>

</xml_diff>